<commit_message>
Add Operation DIRTWERX visual archive display
Embed campaign evidence, expand chapter READMEs, and update navigation, transcriptions, ledgers, and fixity records.
</commit_message>
<xml_diff>
--- a/campaigns/operation-dirtwerx/Operation-DIRTWERX-Campaign-Ledger-v1.0.xlsx
+++ b/campaigns/operation-dirtwerx/Operation-DIRTWERX-Campaign-Ledger-v1.0.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="1" r:id="R7d930f76276a4b99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Ledger" sheetId="2" r:id="R562679afc3f64849"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chronology" sheetId="3" r:id="Re847e88819794bc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Checklist" sheetId="4" r:id="R006e80593a274748"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="1" r:id="Rc8b87d9f36a34ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Ledger" sheetId="2" r:id="Re10f5ff3a7044eed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chronology" sheetId="3" r:id="R577e18b88ade428c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Checklist" sheetId="4" r:id="Rc73fa43d08e3459e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -41,19 +41,8 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -80,59 +69,17 @@
         <x:fgColor rgb="FFFFF0CC"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF3F667A"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF7FAFB"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEAF2F5"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF3F667A"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF7FAFB"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEAF2F5"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="4">
     <x:border/>
     <x:border/>
     <x:border/>
     <x:border/>
-    <x:border/>
-    <x:border/>
-    <x:border/>
-    <x:border/>
-    <x:border>
-      <x:bottom/>
-    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="178">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -331,287 +278,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -844,37 +510,37 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="82" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="3" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="72" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="62" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" hidden="0" customHeight="1">
-      <x:c r="A1" s="145" t="str">
+    <x:row r="1" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A1" s="68" t="str">
         <x:v>#OperationDIRTWERX Campaign Audit Ledger</x:v>
       </x:c>
-      <x:c r="B1" s="145"/>
-      <x:c r="C1" s="145"/>
-      <x:c r="D1" s="145"/>
-      <x:c r="E1" s="145"/>
-      <x:c r="F1" s="147"/>
-      <x:c r="G1" s="147"/>
-      <x:c r="H1" s="147"/>
-    </x:row>
-    <x:row r="2" ht="28" hidden="0" customHeight="1">
-      <x:c r="A2" s="145"/>
-      <x:c r="B2" s="145"/>
-      <x:c r="C2" s="145"/>
-      <x:c r="D2" s="145"/>
-      <x:c r="E2" s="145"/>
-      <x:c r="F2" s="147"/>
-      <x:c r="G2" s="147"/>
-      <x:c r="H2" s="147"/>
+      <x:c r="B1" s="68"/>
+      <x:c r="C1" s="68"/>
+      <x:c r="D1" s="68"/>
+      <x:c r="E1" s="68"/>
+      <x:c r="F1" s="5"/>
+      <x:c r="G1" s="5"/>
+      <x:c r="H1" s="5"/>
+    </x:row>
+    <x:row r="2" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A2" s="68"/>
+      <x:c r="B2" s="68"/>
+      <x:c r="C2" s="68"/>
+      <x:c r="D2" s="68"/>
+      <x:c r="E2" s="68"/>
+      <x:c r="F2" s="5"/>
+      <x:c r="G2" s="5"/>
+      <x:c r="H2" s="5"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="26"/>
@@ -883,165 +549,162 @@
       <x:c r="D3" s="26"/>
       <x:c r="E3" s="26"/>
     </x:row>
-    <x:row r="4" ht="24" hidden="0" customHeight="1">
-      <x:c r="A4" s="88" t="str">
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A4" s="69" t="str">
         <x:v>Metric</x:v>
       </x:c>
-      <x:c r="B4" s="89" t="str">
+      <x:c r="B4" s="69" t="str">
         <x:v>Value</x:v>
       </x:c>
       <x:c r="C4" s="26"/>
-      <x:c r="D4" s="148" t="str">
+      <x:c r="D4" s="81" t="str">
         <x:v>Governing Decisions</x:v>
       </x:c>
-      <x:c r="E4" s="149"/>
-      <x:c r="F4" s="151"/>
-      <x:c r="G4" s="151"/>
-      <x:c r="H4" s="151"/>
-    </x:row>
-    <x:row r="5" ht="32" hidden="0" customHeight="1">
-      <x:c r="A5" s="107" t="str">
+      <x:c r="E4" s="81"/>
+      <x:c r="F4" s="12"/>
+      <x:c r="G4" s="12"/>
+      <x:c r="H4" s="12"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="70" t="str">
         <x:v>Official narrative chapters</x:v>
       </x:c>
-      <x:c r="B5" s="108" t="n">
+      <x:c r="B5" s="58" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C5" s="26"/>
-      <x:c r="D5" s="114" t="str">
+      <x:c r="D5" s="78" t="str">
         <x:v>1.</x:v>
       </x:c>
-      <x:c r="E5" s="108" t="str">
+      <x:c r="E5" s="76" t="str">
         <x:v>Preserve official campaign title, chapter titles, and page sequence.</x:v>
       </x:c>
       <x:c r="F5" s="76"/>
       <x:c r="G5" s="76"/>
       <x:c r="H5" s="76"/>
     </x:row>
-    <x:row r="6" ht="32" hidden="0" customHeight="1">
-      <x:c r="A6" s="107" t="str">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="70" t="str">
         <x:v>Narrative units incl. intro/epilogue</x:v>
       </x:c>
-      <x:c r="B6" s="108" t="n">
+      <x:c r="B6" s="58" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="26"/>
-      <x:c r="D6" s="114" t="str">
+      <x:c r="D6" s="78" t="str">
         <x:v>2.</x:v>
       </x:c>
-      <x:c r="E6" s="108" t="str">
+      <x:c r="E6" s="76" t="str">
         <x:v>Maintain a separate source-publication chronology.</x:v>
       </x:c>
       <x:c r="F6" s="76"/>
       <x:c r="G6" s="76"/>
       <x:c r="H6" s="76"/>
     </x:row>
-    <x:row r="7" ht="32" hidden="0" customHeight="1">
-      <x:c r="A7" s="107" t="str">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="70" t="str">
         <x:v>Supplied source-image records</x:v>
       </x:c>
-      <x:c r="B7" s="108" t="n">
+      <x:c r="B7" s="58" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="C7" s="26"/>
-      <x:c r="D7" s="114" t="str">
+      <x:c r="D7" s="78" t="str">
         <x:v>3.</x:v>
       </x:c>
-      <x:c r="E7" s="108" t="str">
+      <x:c r="E7" s="76" t="str">
         <x:v>Preserve original wording separately from normalized summaries.</x:v>
       </x:c>
       <x:c r="F7" s="76"/>
       <x:c r="G7" s="76"/>
       <x:c r="H7" s="76"/>
     </x:row>
-    <x:row r="8" ht="32" hidden="0" customHeight="1">
-      <x:c r="A8" s="107" t="str">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="70" t="str">
         <x:v>Supplied page-capture images</x:v>
       </x:c>
-      <x:c r="B8" s="108" t="n">
+      <x:c r="B8" s="58" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="C8" s="26"/>
-      <x:c r="D8" s="114" t="str">
+      <x:c r="D8" s="78" t="str">
         <x:v>4.</x:v>
       </x:c>
-      <x:c r="E8" s="108" t="str">
+      <x:c r="E8" s="76" t="str">
         <x:v>Keep the acquisition story offline as the source page directs.</x:v>
       </x:c>
       <x:c r="F8" s="76"/>
       <x:c r="G8" s="76"/>
       <x:c r="H8" s="76"/>
     </x:row>
-    <x:row r="9" ht="32" hidden="0" customHeight="1">
-      <x:c r="A9" s="107" t="str">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="70" t="str">
         <x:v>Dated top-level source posts</x:v>
       </x:c>
-      <x:c r="B9" s="108" t="n">
+      <x:c r="B9" s="58" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C9" s="26"/>
-      <x:c r="D9" s="109" t="str">
+      <x:c r="D9" s="78" t="str">
         <x:v>5.</x:v>
       </x:c>
-      <x:c r="E9" s="115" t="str">
+      <x:c r="E9" s="76" t="str">
         <x:v>Do not fill missing dates, URLs, cropped text, or context from assumption.</x:v>
       </x:c>
       <x:c r="F9" s="76"/>
       <x:c r="G9" s="76"/>
       <x:c r="H9" s="76"/>
     </x:row>
-    <x:row r="10" ht="32" hidden="0" customHeight="1">
-      <x:c r="A10" s="107" t="str">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="26" t="str">
         <x:v>Undated / non-post source records</x:v>
       </x:c>
-      <x:c r="B10" s="108" t="n">
+      <x:c r="B10" s="26" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C10" s="26"/>
       <x:c r="D10" s="26"/>
       <x:c r="E10" s="26"/>
     </x:row>
-    <x:row r="11" ht="32" hidden="0" customHeight="1">
-      <x:c r="A11" s="107" t="str">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="26" t="str">
         <x:v>First page/chronology divergence</x:v>
       </x:c>
-      <x:c r="B11" s="108" t="str">
+      <x:c r="B11" s="26" t="str">
         <x:v>Chapter 2</x:v>
       </x:c>
       <x:c r="C11" s="26"/>
       <x:c r="D11" s="26"/>
       <x:c r="E11" s="26"/>
     </x:row>
-    <x:row r="12" ht="32" hidden="0" customHeight="1">
-      <x:c r="A12" s="153" t="str">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="45" t="str">
         <x:v>Top-level publication span</x:v>
       </x:c>
-      <x:c r="B12" s="159" t="str">
+      <x:c r="B12" s="45" t="str">
         <x:v>April 10-November 27, 2025</x:v>
       </x:c>
-      <x:c r="C12" s="162"/>
-      <x:c r="D12" s="162"/>
-      <x:c r="E12" s="162"/>
-      <x:c r="F12" s="163"/>
-      <x:c r="G12" s="163"/>
-      <x:c r="H12" s="163"/>
-    </x:row>
-    <x:row r="13" ht="24" hidden="0" customHeight="1">
-      <x:c r="A13" s="148" t="str">
+      <x:c r="C12" s="45"/>
+      <x:c r="D12" s="45"/>
+      <x:c r="E12" s="45"/>
+      <x:c r="F12" s="35"/>
+      <x:c r="G12" s="35"/>
+      <x:c r="H12" s="35"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="71" t="str">
         <x:v>Definitive source-publication order</x:v>
       </x:c>
-      <x:c r="B13" s="164"/>
-      <x:c r="C13" s="164"/>
-      <x:c r="D13" s="164"/>
-      <x:c r="E13" s="149"/>
-      <x:c r="F13" s="151"/>
-      <x:c r="G13" s="151"/>
-      <x:c r="H13" s="151"/>
-    </x:row>
-    <x:row r="14" ht="24" hidden="0" customHeight="1">
-      <x:c r="A14" s="88" t="str">
+      <x:c r="B13" s="71"/>
+      <x:c r="C13" s="26"/>
+      <x:c r="D13" s="26"/>
+      <x:c r="E13" s="26"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="52" t="str">
         <x:v>Rank</x:v>
       </x:c>
-      <x:c r="B14" s="89" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>Source / Date</x:v>
       </x:c>
       <x:c r="C14" s="26"/>
@@ -1051,11 +714,11 @@
       <x:c r="G14" s="26"/>
       <x:c r="H14" s="26"/>
     </x:row>
-    <x:row r="15" ht="30" hidden="0" customHeight="1">
-      <x:c r="A15" s="124" t="n">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="52" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B15" s="125" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>2025-04-10 — Source 001: Campaign launch and disassembled-bike documentation</x:v>
       </x:c>
       <x:c r="C15" s="26"/>
@@ -1065,11 +728,11 @@
       <x:c r="G15" s="26"/>
       <x:c r="H15" s="26"/>
     </x:row>
-    <x:row r="16" ht="30" hidden="0" customHeight="1">
-      <x:c r="A16" s="124" t="n">
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="52" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B16" s="125" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>2025-04-15 — Source 014: DIRTWERX story prompt and jersey/helmet display</x:v>
       </x:c>
       <x:c r="C16" s="26"/>
@@ -1079,11 +742,11 @@
       <x:c r="G16" s="26"/>
       <x:c r="H16" s="26"/>
     </x:row>
-    <x:row r="17" ht="30" hidden="0" customHeight="1">
-      <x:c r="A17" s="124" t="n">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="52" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B17" s="125" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>2025-04-25 — Source 003: XL 45 discovery and frame-condition documentation</x:v>
       </x:c>
       <x:c r="C17" s="26"/>
@@ -1093,11 +756,11 @@
       <x:c r="G17" s="26"/>
       <x:c r="H17" s="26"/>
     </x:row>
-    <x:row r="18" ht="30" hidden="0" customHeight="1">
-      <x:c r="A18" s="124" t="n">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="52" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B18" s="125" t="str">
+      <x:c r="B18" s="26" t="str">
         <x:v>2025-04-28 — Source 004: Handlebar straightening before-and-after</x:v>
       </x:c>
       <x:c r="C18" s="26"/>
@@ -1107,11 +770,11 @@
       <x:c r="G18" s="26"/>
       <x:c r="H18" s="26"/>
     </x:row>
-    <x:row r="19" ht="30" hidden="0" customHeight="1">
-      <x:c r="A19" s="124" t="n">
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="52" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B19" s="125" t="str">
+      <x:c r="B19" s="26" t="str">
         <x:v>2025-04-28 — Source 008: Fall Risk Racing care-package support</x:v>
       </x:c>
       <x:c r="C19" s="26"/>
@@ -1121,11 +784,11 @@
       <x:c r="G19" s="26"/>
       <x:c r="H19" s="26"/>
     </x:row>
-    <x:row r="20" ht="30" hidden="0" customHeight="1">
-      <x:c r="A20" s="124" t="n">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="52" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B20" s="125" t="str">
+      <x:c r="B20" s="26" t="str">
         <x:v>2025-05-02 — Source 009: Freewheel preservation prompt</x:v>
       </x:c>
       <x:c r="C20" s="26"/>
@@ -1135,11 +798,11 @@
       <x:c r="G20" s="26"/>
       <x:c r="H20" s="26"/>
     </x:row>
-    <x:row r="21" ht="30" hidden="0" customHeight="1">
-      <x:c r="A21" s="124" t="n">
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="52" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B21" s="125" t="str">
+      <x:c r="B21" s="26" t="str">
         <x:v>2025-05-03 — Source 010: Seat cleaning and clear-sealing documentation</x:v>
       </x:c>
       <x:c r="C21" s="26"/>
@@ -1149,11 +812,11 @@
       <x:c r="G21" s="26"/>
       <x:c r="H21" s="26"/>
     </x:row>
-    <x:row r="22" ht="30" hidden="0" customHeight="1">
-      <x:c r="A22" s="124" t="n">
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="52" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B22" s="125" t="str">
+      <x:c r="B22" s="26" t="str">
         <x:v>2025-05-14 — Source 013: Eddy King pin, toolbox, and DIRTWERX jersey display</x:v>
       </x:c>
       <x:c r="C22" s="26"/>
@@ -1163,11 +826,11 @@
       <x:c r="G22" s="26"/>
       <x:c r="H22" s="26"/>
     </x:row>
-    <x:row r="23" ht="30" hidden="0" customHeight="1">
-      <x:c r="A23" s="124" t="n">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="52" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B23" s="125" t="str">
+      <x:c r="B23" s="26" t="str">
         <x:v>2025-09-02 — Source 012: DIRTWERX painkiller arrival and backstory prompt</x:v>
       </x:c>
       <x:c r="C23" s="26"/>
@@ -1177,11 +840,11 @@
       <x:c r="G23" s="26"/>
       <x:c r="H23" s="26"/>
     </x:row>
-    <x:row r="24" ht="30" hidden="0" customHeight="1">
-      <x:c r="A24" s="126" t="n">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="52" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B24" s="127" t="str">
+      <x:c r="B24" s="26" t="str">
         <x:v>2025-11-27 — Source 002: Completed bicycle returned to the Leary family</x:v>
       </x:c>
       <x:c r="C24" s="26"/>
@@ -1191,45 +854,45 @@
       <x:c r="G24" s="26"/>
       <x:c r="H24" s="26"/>
     </x:row>
-    <x:row r="25" ht="46" hidden="0" customHeight="1">
-      <x:c r="A25" s="174" t="str">
+    <x:row r="25" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A25" s="52" t="str">
         <x:v>Unplaced: Sources 005-006 — memorial-card images; publication/capture dates not supplied.</x:v>
       </x:c>
-      <x:c r="B25" s="174"/>
-      <x:c r="C25" s="174"/>
-      <x:c r="D25" s="174"/>
-      <x:c r="E25" s="174"/>
-      <x:c r="F25" s="174"/>
-      <x:c r="G25" s="174"/>
-      <x:c r="H25" s="174"/>
-    </x:row>
-    <x:row r="26" ht="46" hidden="0" customHeight="1">
-      <x:c r="A26" s="174" t="str">
+      <x:c r="B25" s="26"/>
+      <x:c r="C25" s="26"/>
+      <x:c r="D25" s="26"/>
+      <x:c r="E25" s="26"/>
+      <x:c r="F25" s="26"/>
+      <x:c r="G25" s="26"/>
+      <x:c r="H25" s="26"/>
+    </x:row>
+    <x:row r="26" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A26" s="52" t="str">
         <x:v>Unplaced: Source 007 — Justin Dumas post; only relative timestamp “4h” visible.</x:v>
       </x:c>
-      <x:c r="B26" s="174"/>
-      <x:c r="C26" s="174"/>
-      <x:c r="D26" s="174"/>
-      <x:c r="E26" s="174"/>
-      <x:c r="F26" s="174"/>
-      <x:c r="G26" s="174"/>
-      <x:c r="H26" s="174"/>
-    </x:row>
-    <x:row r="27" ht="46" hidden="0" customHeight="1">
-      <x:c r="A27" s="174" t="str">
+      <x:c r="B26" s="26"/>
+      <x:c r="C26" s="26"/>
+      <x:c r="D26" s="26"/>
+      <x:c r="E26" s="26"/>
+      <x:c r="F26" s="26"/>
+      <x:c r="G26" s="26"/>
+      <x:c r="H26" s="26"/>
+    </x:row>
+    <x:row r="27" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A27" s="52" t="str">
         <x:v>Unplaced: Source 011 — campaign photograph; original capture date/provenance not supplied.</x:v>
       </x:c>
-      <x:c r="B27" s="174"/>
-      <x:c r="C27" s="174"/>
-      <x:c r="D27" s="174"/>
-      <x:c r="E27" s="174"/>
-      <x:c r="F27" s="174"/>
-      <x:c r="G27" s="174"/>
-      <x:c r="H27" s="174"/>
-    </x:row>
-    <x:row r="28" ht="46" hidden="0" customHeight="1">
-      <x:c r="A28" s="136"/>
-      <x:c r="B28" s="137"/>
+      <x:c r="B27" s="26"/>
+      <x:c r="C27" s="26"/>
+      <x:c r="D27" s="26"/>
+      <x:c r="E27" s="26"/>
+      <x:c r="F27" s="26"/>
+      <x:c r="G27" s="26"/>
+      <x:c r="H27" s="26"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="52"/>
+      <x:c r="B28" s="26"/>
       <x:c r="C28" s="26"/>
       <x:c r="D28" s="26"/>
       <x:c r="E28" s="26"/>
@@ -1237,17 +900,17 @@
       <x:c r="G28" s="26"/>
       <x:c r="H28" s="26"/>
     </x:row>
-    <x:row r="29" ht="46" hidden="0" customHeight="1">
-      <x:c r="A29" s="174" t="str">
+    <x:row r="29" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A29" s="52" t="str">
         <x:v>Embedded earlier record: Source 014 contains a Lititz BMX post dated 2025-04-06 inside an April 15 share.</x:v>
       </x:c>
-      <x:c r="B29" s="174"/>
-      <x:c r="C29" s="174"/>
-      <x:c r="D29" s="174"/>
-      <x:c r="E29" s="174"/>
-      <x:c r="F29" s="174"/>
-      <x:c r="G29" s="174"/>
-      <x:c r="H29" s="174"/>
+      <x:c r="B29" s="26"/>
+      <x:c r="C29" s="26"/>
+      <x:c r="D29" s="26"/>
+      <x:c r="E29" s="26"/>
+      <x:c r="F29" s="26"/>
+      <x:c r="G29" s="26"/>
+      <x:c r="H29" s="26"/>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="52"/>
@@ -1281,6 +944,9 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="D4:H4"/>
+    <x:mergeCell ref="A12:H12"/>
     <x:mergeCell ref="B14:H14"/>
     <x:mergeCell ref="B15:H15"/>
     <x:mergeCell ref="B16:H16"/>
@@ -1292,7 +958,11 @@
     <x:mergeCell ref="B22:H22"/>
     <x:mergeCell ref="B23:H23"/>
     <x:mergeCell ref="B24:H24"/>
+    <x:mergeCell ref="B25:H25"/>
+    <x:mergeCell ref="B26:H26"/>
+    <x:mergeCell ref="B27:H27"/>
     <x:mergeCell ref="B28:H28"/>
+    <x:mergeCell ref="B29:H29"/>
     <x:mergeCell ref="B30:H30"/>
     <x:mergeCell ref="B31:H31"/>
     <x:mergeCell ref="A32:H32"/>
@@ -1301,14 +971,6 @@
     <x:mergeCell ref="E7:H7"/>
     <x:mergeCell ref="E8:H8"/>
     <x:mergeCell ref="E9:H9"/>
-    <x:mergeCell ref="A1:H2"/>
-    <x:mergeCell ref="D4:H4"/>
-    <x:mergeCell ref="B12:H12"/>
-    <x:mergeCell ref="A13:H13"/>
-    <x:mergeCell ref="A25:H25"/>
-    <x:mergeCell ref="A26:H26"/>
-    <x:mergeCell ref="A27:H27"/>
-    <x:mergeCell ref="A29:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1827,7 +1489,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3348971d5f5449ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R020d0bb5be8344b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2181,7 +1843,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R124b55cd8fb5457f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f1cdf50dcb144ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2592,7 +2254,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dd03ad4e9304a70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a63bde430cf493d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>